<commit_message>
RT21 export: add Combined pivot sheet + throttling/lock hardening
- New 5th sheet 'Combined' merging order and invoice Item lines for
  pivoting: SO Number (Order_No fallback invoice no), Status
  (Open/Released/Invoiced), No, Description, Quantity (outstanding for
  open orders to avoid double counting), Unit Price (computed for order
  lines), Line_Amount, Sell_to_Customer_No/Name.
- Template regenerated with the Combined sheet.
- All Graph nodes now retry (5x, 5s) to ride out 429 throttling.
- New 'Ensure Sheets' loop adds any missing worksheet after the
  template copy, so a locked file (423) can no longer cause a 404 on
  write. Client secret redacted in repo copy; live value set in n8n.
</commit_message>
<xml_diff>
--- a/n8n/templates/RT21_Orders_and_Invoices_template.xlsx
+++ b/n8n/templates/RT21_Orders_and_Invoices_template.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Order Lines" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Invoices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Invoice Lines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Combined" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,4 +461,17 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>